<commit_message>
add system modelling. Add arduino script for calc of digital control loop timing
</commit_message>
<xml_diff>
--- a/background/TheoreticalPlots/hallSensorReadings.xlsx
+++ b/background/TheoreticalPlots/hallSensorReadings.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Daniel\Documents\Personal Projects\Leviosa\background\TheoreticalPlots\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22859989-64B4-4676-9813-0467ACBEE6D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E48548E-8783-40DF-81FC-AB8E3FC92DE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{70F60A36-1F6A-4137-A42D-DB1ECF4242FE}"/>
   </bookViews>
@@ -6979,8 +6979,8 @@
     <xdr:to>
       <xdr:col>36</xdr:col>
       <xdr:colOff>200320</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>79342</xdr:rowOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>147484</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>

</xml_diff>